<commit_message>
Updated POL_grids_kan model - 2026-06-05 12:28
</commit_message>
<xml_diff>
--- a/VerveStacks_POL_grids_kan/Sets-vervestacks.xlsx
+++ b/VerveStacks_POL_grids_kan/Sets-vervestacks.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr updateLinks="never" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_POL_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D3A3A43F-A398-4060-BD4A-DD633B820387}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{028518FF-1208-4FD7-B2AE-5C53BA952015}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1052" uniqueCount="570">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1220" uniqueCount="654">
   <si>
     <t>~TFM_Psets</t>
   </si>
@@ -349,1405 +349,1657 @@
     <t>t_pos_andor</t>
   </si>
   <si>
-    <t>p_PL1</t>
-  </si>
-  <si>
-    <t>e_PL1*</t>
+    <t>p_PL1-400_POL</t>
+  </si>
+  <si>
+    <t>e_PL1-400_POL*</t>
   </si>
   <si>
     <t>OR</t>
   </si>
   <si>
-    <t>p_PL10</t>
-  </si>
-  <si>
-    <t>e_PL10*</t>
-  </si>
-  <si>
-    <t>p_PL11</t>
-  </si>
-  <si>
-    <t>e_PL11*</t>
-  </si>
-  <si>
-    <t>p_PL13</t>
-  </si>
-  <si>
-    <t>e_PL13*</t>
-  </si>
-  <si>
-    <t>p_PL14</t>
-  </si>
-  <si>
-    <t>e_PL14*</t>
-  </si>
-  <si>
-    <t>p_PL15</t>
-  </si>
-  <si>
-    <t>e_PL15*</t>
-  </si>
-  <si>
-    <t>p_PL16</t>
-  </si>
-  <si>
-    <t>e_PL16*</t>
-  </si>
-  <si>
-    <t>p_PL17</t>
-  </si>
-  <si>
-    <t>e_PL17*</t>
-  </si>
-  <si>
-    <t>p_PL18</t>
-  </si>
-  <si>
-    <t>e_PL18*</t>
-  </si>
-  <si>
-    <t>p_PL19</t>
-  </si>
-  <si>
-    <t>e_PL19*</t>
-  </si>
-  <si>
-    <t>p_PL2</t>
-  </si>
-  <si>
-    <t>e_PL2*</t>
-  </si>
-  <si>
-    <t>p_PL20</t>
-  </si>
-  <si>
-    <t>e_PL20*</t>
-  </si>
-  <si>
-    <t>p_PL21</t>
-  </si>
-  <si>
-    <t>e_PL21*</t>
-  </si>
-  <si>
-    <t>p_PL22</t>
-  </si>
-  <si>
-    <t>e_PL22*</t>
-  </si>
-  <si>
-    <t>p_PL23</t>
-  </si>
-  <si>
-    <t>e_PL23*</t>
-  </si>
-  <si>
-    <t>p_PL24</t>
-  </si>
-  <si>
-    <t>e_PL24*</t>
-  </si>
-  <si>
-    <t>p_PL25</t>
-  </si>
-  <si>
-    <t>e_PL25*</t>
-  </si>
-  <si>
-    <t>p_PL26</t>
-  </si>
-  <si>
-    <t>e_PL26*</t>
-  </si>
-  <si>
-    <t>p_PL27</t>
-  </si>
-  <si>
-    <t>e_PL27*</t>
-  </si>
-  <si>
-    <t>p_PL28</t>
-  </si>
-  <si>
-    <t>e_PL28*</t>
-  </si>
-  <si>
-    <t>p_PL29</t>
-  </si>
-  <si>
-    <t>e_PL29*</t>
-  </si>
-  <si>
-    <t>p_PL3</t>
-  </si>
-  <si>
-    <t>e_PL3*</t>
-  </si>
-  <si>
-    <t>p_PL30</t>
-  </si>
-  <si>
-    <t>e_PL30*</t>
-  </si>
-  <si>
-    <t>p_PL31</t>
-  </si>
-  <si>
-    <t>e_PL31*</t>
-  </si>
-  <si>
-    <t>p_PL32</t>
-  </si>
-  <si>
-    <t>e_PL32*</t>
-  </si>
-  <si>
-    <t>p_PL33</t>
-  </si>
-  <si>
-    <t>e_PL33*</t>
-  </si>
-  <si>
-    <t>p_PL34</t>
-  </si>
-  <si>
-    <t>e_PL34*</t>
-  </si>
-  <si>
-    <t>p_PL35</t>
-  </si>
-  <si>
-    <t>e_PL35*</t>
-  </si>
-  <si>
-    <t>p_PL36</t>
-  </si>
-  <si>
-    <t>e_PL36*</t>
-  </si>
-  <si>
-    <t>p_PL37</t>
-  </si>
-  <si>
-    <t>e_PL37*</t>
-  </si>
-  <si>
-    <t>p_PL38</t>
-  </si>
-  <si>
-    <t>e_PL38*</t>
-  </si>
-  <si>
-    <t>p_PL39</t>
-  </si>
-  <si>
-    <t>e_PL39*</t>
-  </si>
-  <si>
-    <t>p_PL4</t>
-  </si>
-  <si>
-    <t>e_PL4*</t>
-  </si>
-  <si>
-    <t>p_PL40</t>
-  </si>
-  <si>
-    <t>e_PL40*</t>
-  </si>
-  <si>
-    <t>p_PL41</t>
-  </si>
-  <si>
-    <t>e_PL41*</t>
-  </si>
-  <si>
-    <t>p_PL42</t>
-  </si>
-  <si>
-    <t>e_PL42*</t>
-  </si>
-  <si>
-    <t>p_PL43</t>
-  </si>
-  <si>
-    <t>e_PL43*</t>
-  </si>
-  <si>
-    <t>p_PL44</t>
-  </si>
-  <si>
-    <t>e_PL44*</t>
-  </si>
-  <si>
-    <t>p_PL45</t>
-  </si>
-  <si>
-    <t>e_PL45*</t>
-  </si>
-  <si>
-    <t>p_PL46</t>
-  </si>
-  <si>
-    <t>e_PL46*</t>
-  </si>
-  <si>
-    <t>p_PL47</t>
-  </si>
-  <si>
-    <t>e_PL47*</t>
-  </si>
-  <si>
-    <t>p_PL48</t>
-  </si>
-  <si>
-    <t>e_PL48*</t>
-  </si>
-  <si>
-    <t>p_PL49</t>
-  </si>
-  <si>
-    <t>e_PL49*</t>
-  </si>
-  <si>
-    <t>p_PL5</t>
-  </si>
-  <si>
-    <t>e_PL5*</t>
-  </si>
-  <si>
-    <t>p_PL50</t>
-  </si>
-  <si>
-    <t>e_PL50*</t>
-  </si>
-  <si>
-    <t>p_PL51</t>
-  </si>
-  <si>
-    <t>e_PL51*</t>
-  </si>
-  <si>
-    <t>p_PL52</t>
-  </si>
-  <si>
-    <t>e_PL52*</t>
-  </si>
-  <si>
-    <t>p_PL53</t>
-  </si>
-  <si>
-    <t>e_PL53*</t>
-  </si>
-  <si>
-    <t>p_PL54</t>
-  </si>
-  <si>
-    <t>e_PL54*</t>
-  </si>
-  <si>
-    <t>p_PL55</t>
-  </si>
-  <si>
-    <t>e_PL55*</t>
-  </si>
-  <si>
-    <t>p_PL56</t>
-  </si>
-  <si>
-    <t>e_PL56*</t>
-  </si>
-  <si>
-    <t>p_PL57</t>
-  </si>
-  <si>
-    <t>e_PL57*</t>
-  </si>
-  <si>
-    <t>p_PL58</t>
-  </si>
-  <si>
-    <t>e_PL58*</t>
-  </si>
-  <si>
-    <t>p_PL59</t>
-  </si>
-  <si>
-    <t>e_PL59*</t>
-  </si>
-  <si>
-    <t>p_PL6</t>
-  </si>
-  <si>
-    <t>e_PL6*</t>
-  </si>
-  <si>
-    <t>p_PL60</t>
-  </si>
-  <si>
-    <t>e_PL60*</t>
-  </si>
-  <si>
-    <t>p_PL61</t>
-  </si>
-  <si>
-    <t>e_PL61*</t>
-  </si>
-  <si>
-    <t>p_PL62</t>
-  </si>
-  <si>
-    <t>e_PL62*</t>
-  </si>
-  <si>
-    <t>p_PL7</t>
-  </si>
-  <si>
-    <t>e_PL7*</t>
-  </si>
-  <si>
-    <t>p_PL8</t>
-  </si>
-  <si>
-    <t>e_PL8*</t>
-  </si>
-  <si>
-    <t>p_r18085709</t>
-  </si>
-  <si>
-    <t>e_r18085709*</t>
-  </si>
-  <si>
-    <t>p_r9399771</t>
-  </si>
-  <si>
-    <t>e_r9399771*</t>
-  </si>
-  <si>
-    <t>p_w101914781</t>
-  </si>
-  <si>
-    <t>e_w101914781*</t>
-  </si>
-  <si>
-    <t>p_w101915790</t>
-  </si>
-  <si>
-    <t>e_w101915790*</t>
-  </si>
-  <si>
-    <t>p_w101982559</t>
-  </si>
-  <si>
-    <t>e_w101982559*</t>
-  </si>
-  <si>
-    <t>p_w102165724</t>
-  </si>
-  <si>
-    <t>e_w102165724*</t>
-  </si>
-  <si>
-    <t>p_w1022342082</t>
-  </si>
-  <si>
-    <t>e_w1022342082*</t>
-  </si>
-  <si>
-    <t>p_w111615226</t>
-  </si>
-  <si>
-    <t>e_w111615226*</t>
-  </si>
-  <si>
-    <t>p_w112614319</t>
-  </si>
-  <si>
-    <t>e_w112614319*</t>
-  </si>
-  <si>
-    <t>p_w115801644</t>
-  </si>
-  <si>
-    <t>e_w115801644*</t>
-  </si>
-  <si>
-    <t>p_w121656686</t>
-  </si>
-  <si>
-    <t>e_w121656686*</t>
-  </si>
-  <si>
-    <t>p_w130644710</t>
-  </si>
-  <si>
-    <t>e_w130644710*</t>
-  </si>
-  <si>
-    <t>p_w131120723</t>
-  </si>
-  <si>
-    <t>e_w131120723*</t>
-  </si>
-  <si>
-    <t>p_w133537926</t>
-  </si>
-  <si>
-    <t>e_w133537926*</t>
-  </si>
-  <si>
-    <t>p_w135598292</t>
-  </si>
-  <si>
-    <t>e_w135598292*</t>
-  </si>
-  <si>
-    <t>p_w139452056</t>
-  </si>
-  <si>
-    <t>e_w139452056*</t>
-  </si>
-  <si>
-    <t>p_w143484238</t>
-  </si>
-  <si>
-    <t>e_w143484238*</t>
-  </si>
-  <si>
-    <t>p_w144646702</t>
-  </si>
-  <si>
-    <t>e_w144646702*</t>
-  </si>
-  <si>
-    <t>p_w145037309</t>
-  </si>
-  <si>
-    <t>e_w145037309*</t>
-  </si>
-  <si>
-    <t>p_w148060965</t>
-  </si>
-  <si>
-    <t>e_w148060965*</t>
-  </si>
-  <si>
-    <t>p_w148197330</t>
-  </si>
-  <si>
-    <t>e_w148197330*</t>
-  </si>
-  <si>
-    <t>p_w153838553</t>
-  </si>
-  <si>
-    <t>e_w153838553*</t>
-  </si>
-  <si>
-    <t>p_w154510504</t>
-  </si>
-  <si>
-    <t>e_w154510504*</t>
-  </si>
-  <si>
-    <t>p_w154894455</t>
-  </si>
-  <si>
-    <t>e_w154894455*</t>
-  </si>
-  <si>
-    <t>p_w155971668</t>
-  </si>
-  <si>
-    <t>e_w155971668*</t>
-  </si>
-  <si>
-    <t>p_w158232924</t>
-  </si>
-  <si>
-    <t>e_w158232924*</t>
-  </si>
-  <si>
-    <t>p_w165763717</t>
-  </si>
-  <si>
-    <t>e_w165763717*</t>
-  </si>
-  <si>
-    <t>p_w166710856</t>
-  </si>
-  <si>
-    <t>e_w166710856*</t>
-  </si>
-  <si>
-    <t>p_w166838338</t>
-  </si>
-  <si>
-    <t>e_w166838338*</t>
-  </si>
-  <si>
-    <t>p_w170249563</t>
-  </si>
-  <si>
-    <t>e_w170249563*</t>
-  </si>
-  <si>
-    <t>p_w170259740</t>
-  </si>
-  <si>
-    <t>e_w170259740*</t>
-  </si>
-  <si>
-    <t>p_w170316833</t>
-  </si>
-  <si>
-    <t>e_w170316833*</t>
-  </si>
-  <si>
-    <t>p_w170368942</t>
-  </si>
-  <si>
-    <t>e_w170368942*</t>
-  </si>
-  <si>
-    <t>p_w171383831</t>
-  </si>
-  <si>
-    <t>e_w171383831*</t>
-  </si>
-  <si>
-    <t>p_w171917072</t>
-  </si>
-  <si>
-    <t>e_w171917072*</t>
-  </si>
-  <si>
-    <t>p_w171992870</t>
-  </si>
-  <si>
-    <t>e_w171992870*</t>
-  </si>
-  <si>
-    <t>p_w173582810</t>
-  </si>
-  <si>
-    <t>e_w173582810*</t>
-  </si>
-  <si>
-    <t>p_w173613665</t>
-  </si>
-  <si>
-    <t>e_w173613665*</t>
-  </si>
-  <si>
-    <t>p_w175406958</t>
-  </si>
-  <si>
-    <t>e_w175406958*</t>
-  </si>
-  <si>
-    <t>p_w177749653</t>
-  </si>
-  <si>
-    <t>e_w177749653*</t>
-  </si>
-  <si>
-    <t>p_w178756295</t>
-  </si>
-  <si>
-    <t>e_w178756295*</t>
-  </si>
-  <si>
-    <t>p_w178838661</t>
-  </si>
-  <si>
-    <t>e_w178838661*</t>
-  </si>
-  <si>
-    <t>p_w179279860</t>
-  </si>
-  <si>
-    <t>e_w179279860*</t>
-  </si>
-  <si>
-    <t>p_w180535363</t>
-  </si>
-  <si>
-    <t>e_w180535363*</t>
-  </si>
-  <si>
-    <t>p_w180542657</t>
-  </si>
-  <si>
-    <t>e_w180542657*</t>
-  </si>
-  <si>
-    <t>p_w183259405</t>
-  </si>
-  <si>
-    <t>e_w183259405*</t>
-  </si>
-  <si>
-    <t>p_w183945016</t>
-  </si>
-  <si>
-    <t>e_w183945016*</t>
-  </si>
-  <si>
-    <t>p_w184899160</t>
-  </si>
-  <si>
-    <t>e_w184899160*</t>
-  </si>
-  <si>
-    <t>p_w185454704</t>
-  </si>
-  <si>
-    <t>e_w185454704*</t>
-  </si>
-  <si>
-    <t>p_w185459155</t>
-  </si>
-  <si>
-    <t>e_w185459155*</t>
-  </si>
-  <si>
-    <t>p_w189501431</t>
-  </si>
-  <si>
-    <t>e_w189501431*</t>
-  </si>
-  <si>
-    <t>p_w189851841</t>
-  </si>
-  <si>
-    <t>e_w189851841*</t>
-  </si>
-  <si>
-    <t>p_w191035265</t>
-  </si>
-  <si>
-    <t>e_w191035265*</t>
-  </si>
-  <si>
-    <t>p_w191038569</t>
-  </si>
-  <si>
-    <t>e_w191038569*</t>
-  </si>
-  <si>
-    <t>p_w191352746</t>
-  </si>
-  <si>
-    <t>e_w191352746*</t>
-  </si>
-  <si>
-    <t>p_w194903381</t>
-  </si>
-  <si>
-    <t>e_w194903381*</t>
-  </si>
-  <si>
-    <t>p_w198635989</t>
-  </si>
-  <si>
-    <t>e_w198635989*</t>
-  </si>
-  <si>
-    <t>p_w199098050</t>
-  </si>
-  <si>
-    <t>e_w199098050*</t>
-  </si>
-  <si>
-    <t>p_w199098053</t>
-  </si>
-  <si>
-    <t>e_w199098053*</t>
-  </si>
-  <si>
-    <t>p_w199098055</t>
-  </si>
-  <si>
-    <t>e_w199098055*</t>
-  </si>
-  <si>
-    <t>p_w215282393</t>
-  </si>
-  <si>
-    <t>e_w215282393*</t>
-  </si>
-  <si>
-    <t>p_w216060722</t>
-  </si>
-  <si>
-    <t>e_w216060722*</t>
-  </si>
-  <si>
-    <t>p_w216975352</t>
-  </si>
-  <si>
-    <t>e_w216975352*</t>
-  </si>
-  <si>
-    <t>p_w217899005</t>
-  </si>
-  <si>
-    <t>e_w217899005*</t>
-  </si>
-  <si>
-    <t>p_w224727316</t>
-  </si>
-  <si>
-    <t>e_w224727316*</t>
-  </si>
-  <si>
-    <t>p_w228154083</t>
-  </si>
-  <si>
-    <t>e_w228154083*</t>
-  </si>
-  <si>
-    <t>p_w238640596</t>
-  </si>
-  <si>
-    <t>e_w238640596*</t>
-  </si>
-  <si>
-    <t>p_w241842600</t>
-  </si>
-  <si>
-    <t>e_w241842600*</t>
-  </si>
-  <si>
-    <t>p_w245964556</t>
-  </si>
-  <si>
-    <t>e_w245964556*</t>
-  </si>
-  <si>
-    <t>p_w251239544</t>
-  </si>
-  <si>
-    <t>e_w251239544*</t>
-  </si>
-  <si>
-    <t>p_w254235846</t>
-  </si>
-  <si>
-    <t>e_w254235846*</t>
-  </si>
-  <si>
-    <t>p_w254938713</t>
-  </si>
-  <si>
-    <t>e_w254938713*</t>
-  </si>
-  <si>
-    <t>p_w255232597</t>
-  </si>
-  <si>
-    <t>e_w255232597*</t>
-  </si>
-  <si>
-    <t>p_w255277953</t>
-  </si>
-  <si>
-    <t>e_w255277953*</t>
-  </si>
-  <si>
-    <t>p_w255284259</t>
-  </si>
-  <si>
-    <t>e_w255284259*</t>
-  </si>
-  <si>
-    <t>p_w255293400</t>
-  </si>
-  <si>
-    <t>e_w255293400*</t>
-  </si>
-  <si>
-    <t>p_w255293403</t>
-  </si>
-  <si>
-    <t>e_w255293403*</t>
-  </si>
-  <si>
-    <t>p_w255314292</t>
-  </si>
-  <si>
-    <t>e_w255314292*</t>
-  </si>
-  <si>
-    <t>p_w255972326</t>
-  </si>
-  <si>
-    <t>e_w255972326*</t>
-  </si>
-  <si>
-    <t>p_w255972397</t>
-  </si>
-  <si>
-    <t>e_w255972397*</t>
-  </si>
-  <si>
-    <t>p_w255973806</t>
-  </si>
-  <si>
-    <t>e_w255973806*</t>
-  </si>
-  <si>
-    <t>p_w25898810</t>
-  </si>
-  <si>
-    <t>e_w25898810*</t>
-  </si>
-  <si>
-    <t>p_w276291999</t>
-  </si>
-  <si>
-    <t>e_w276291999*</t>
-  </si>
-  <si>
-    <t>p_w29098336</t>
-  </si>
-  <si>
-    <t>e_w29098336*</t>
-  </si>
-  <si>
-    <t>p_w29115701</t>
-  </si>
-  <si>
-    <t>e_w29115701*</t>
-  </si>
-  <si>
-    <t>p_w291375946</t>
-  </si>
-  <si>
-    <t>e_w291375946*</t>
-  </si>
-  <si>
-    <t>p_w29139402</t>
-  </si>
-  <si>
-    <t>e_w29139402*</t>
-  </si>
-  <si>
-    <t>p_w293484891</t>
-  </si>
-  <si>
-    <t>e_w293484891*</t>
-  </si>
-  <si>
-    <t>p_w293484894</t>
-  </si>
-  <si>
-    <t>e_w293484894*</t>
-  </si>
-  <si>
-    <t>p_w293489607</t>
-  </si>
-  <si>
-    <t>e_w293489607*</t>
-  </si>
-  <si>
-    <t>p_w293489663</t>
-  </si>
-  <si>
-    <t>e_w293489663*</t>
-  </si>
-  <si>
-    <t>p_w303870256</t>
-  </si>
-  <si>
-    <t>e_w303870256*</t>
-  </si>
-  <si>
-    <t>p_w32036484</t>
-  </si>
-  <si>
-    <t>e_w32036484*</t>
-  </si>
-  <si>
-    <t>p_w32943179</t>
-  </si>
-  <si>
-    <t>e_w32943179*</t>
-  </si>
-  <si>
-    <t>p_w336990960</t>
-  </si>
-  <si>
-    <t>e_w336990960*</t>
-  </si>
-  <si>
-    <t>p_w35366436</t>
-  </si>
-  <si>
-    <t>e_w35366436*</t>
-  </si>
-  <si>
-    <t>p_w385098015</t>
-  </si>
-  <si>
-    <t>e_w385098015*</t>
-  </si>
-  <si>
-    <t>p_w385118244</t>
-  </si>
-  <si>
-    <t>e_w385118244*</t>
-  </si>
-  <si>
-    <t>p_w385539724</t>
-  </si>
-  <si>
-    <t>e_w385539724*</t>
-  </si>
-  <si>
-    <t>p_w39428977</t>
-  </si>
-  <si>
-    <t>e_w39428977*</t>
-  </si>
-  <si>
-    <t>p_w40062974</t>
-  </si>
-  <si>
-    <t>e_w40062974*</t>
-  </si>
-  <si>
-    <t>p_w40946784</t>
-  </si>
-  <si>
-    <t>e_w40946784*</t>
-  </si>
-  <si>
-    <t>p_w40946790</t>
-  </si>
-  <si>
-    <t>e_w40946790*</t>
-  </si>
-  <si>
-    <t>p_w44389929</t>
-  </si>
-  <si>
-    <t>e_w44389929*</t>
-  </si>
-  <si>
-    <t>p_w46092396</t>
-  </si>
-  <si>
-    <t>e_w46092396*</t>
-  </si>
-  <si>
-    <t>p_w46235456</t>
-  </si>
-  <si>
-    <t>e_w46235456*</t>
-  </si>
-  <si>
-    <t>p_w534238983</t>
-  </si>
-  <si>
-    <t>e_w534238983*</t>
-  </si>
-  <si>
-    <t>p_w658600169</t>
-  </si>
-  <si>
-    <t>e_w658600169*</t>
-  </si>
-  <si>
-    <t>p_w66051759</t>
-  </si>
-  <si>
-    <t>e_w66051759*</t>
-  </si>
-  <si>
-    <t>p_w66161634</t>
-  </si>
-  <si>
-    <t>e_w66161634*</t>
-  </si>
-  <si>
-    <t>p_w668348943</t>
-  </si>
-  <si>
-    <t>e_w668348943*</t>
-  </si>
-  <si>
-    <t>p_w681264796</t>
-  </si>
-  <si>
-    <t>e_w681264796*</t>
-  </si>
-  <si>
-    <t>p_w726776987</t>
-  </si>
-  <si>
-    <t>e_w726776987*</t>
-  </si>
-  <si>
-    <t>p_w72879943</t>
-  </si>
-  <si>
-    <t>e_w72879943*</t>
-  </si>
-  <si>
-    <t>p_w79033485</t>
-  </si>
-  <si>
-    <t>e_w79033485*</t>
-  </si>
-  <si>
-    <t>p_w86494356</t>
-  </si>
-  <si>
-    <t>e_w86494356*</t>
-  </si>
-  <si>
-    <t>p_w87667718</t>
-  </si>
-  <si>
-    <t>e_w87667718*</t>
-  </si>
-  <si>
-    <t>p_w88544449</t>
-  </si>
-  <si>
-    <t>e_w88544449*</t>
-  </si>
-  <si>
-    <t>p_w89434732</t>
-  </si>
-  <si>
-    <t>e_w89434732*</t>
-  </si>
-  <si>
-    <t>p_w91384044</t>
-  </si>
-  <si>
-    <t>e_w91384044*</t>
-  </si>
-  <si>
-    <t>p_w98611253</t>
-  </si>
-  <si>
-    <t>e_w98611253*</t>
-  </si>
-  <si>
-    <t>p_w98634956</t>
-  </si>
-  <si>
-    <t>e_w98634956*</t>
-  </si>
-  <si>
-    <t>p_w99593626</t>
-  </si>
-  <si>
-    <t>e_w99593626*</t>
-  </si>
-  <si>
-    <t>rez_spv_001</t>
-  </si>
-  <si>
-    <t>elc_spv_001</t>
-  </si>
-  <si>
-    <t>rez_spv_002</t>
-  </si>
-  <si>
-    <t>elc_spv_002</t>
-  </si>
-  <si>
-    <t>rez_spv_003</t>
-  </si>
-  <si>
-    <t>elc_spv_003</t>
-  </si>
-  <si>
-    <t>rez_spv_004</t>
-  </si>
-  <si>
-    <t>elc_spv_004</t>
-  </si>
-  <si>
-    <t>rez_spv_005</t>
-  </si>
-  <si>
-    <t>elc_spv_005</t>
-  </si>
-  <si>
-    <t>rez_spv_006</t>
-  </si>
-  <si>
-    <t>elc_spv_006</t>
-  </si>
-  <si>
-    <t>rez_spv_007</t>
-  </si>
-  <si>
-    <t>elc_spv_007</t>
-  </si>
-  <si>
-    <t>rez_spv_008</t>
-  </si>
-  <si>
-    <t>elc_spv_008</t>
-  </si>
-  <si>
-    <t>rez_spv_009</t>
-  </si>
-  <si>
-    <t>elc_spv_009</t>
-  </si>
-  <si>
-    <t>rez_spv_010</t>
-  </si>
-  <si>
-    <t>elc_spv_010</t>
-  </si>
-  <si>
-    <t>rez_spv_011</t>
-  </si>
-  <si>
-    <t>elc_spv_011</t>
-  </si>
-  <si>
-    <t>rez_spv_012</t>
-  </si>
-  <si>
-    <t>elc_spv_012</t>
-  </si>
-  <si>
-    <t>rez_spv_013</t>
-  </si>
-  <si>
-    <t>elc_spv_013</t>
-  </si>
-  <si>
-    <t>rez_spv_014</t>
-  </si>
-  <si>
-    <t>elc_spv_014</t>
-  </si>
-  <si>
-    <t>rez_spv_015</t>
-  </si>
-  <si>
-    <t>elc_spv_015</t>
-  </si>
-  <si>
-    <t>rez_spv_016</t>
-  </si>
-  <si>
-    <t>elc_spv_016</t>
-  </si>
-  <si>
-    <t>rez_spv_017</t>
-  </si>
-  <si>
-    <t>elc_spv_017</t>
-  </si>
-  <si>
-    <t>rez_spv_018</t>
-  </si>
-  <si>
-    <t>elc_spv_018</t>
-  </si>
-  <si>
-    <t>rez_spv_019</t>
-  </si>
-  <si>
-    <t>elc_spv_019</t>
-  </si>
-  <si>
-    <t>rez_spv_020</t>
-  </si>
-  <si>
-    <t>elc_spv_020</t>
-  </si>
-  <si>
-    <t>rez_won_001</t>
-  </si>
-  <si>
-    <t>elc_won_001</t>
-  </si>
-  <si>
-    <t>rez_won_002</t>
-  </si>
-  <si>
-    <t>elc_won_002</t>
-  </si>
-  <si>
-    <t>rez_won_003</t>
-  </si>
-  <si>
-    <t>elc_won_003</t>
-  </si>
-  <si>
-    <t>rez_won_004</t>
-  </si>
-  <si>
-    <t>elc_won_004</t>
-  </si>
-  <si>
-    <t>rez_won_005</t>
-  </si>
-  <si>
-    <t>elc_won_005</t>
-  </si>
-  <si>
-    <t>rez_won_006</t>
-  </si>
-  <si>
-    <t>elc_won_006</t>
-  </si>
-  <si>
-    <t>rez_won_007</t>
-  </si>
-  <si>
-    <t>elc_won_007</t>
-  </si>
-  <si>
-    <t>rez_won_008</t>
-  </si>
-  <si>
-    <t>elc_won_008</t>
-  </si>
-  <si>
-    <t>rez_won_009</t>
-  </si>
-  <si>
-    <t>elc_won_009</t>
-  </si>
-  <si>
-    <t>rez_won_010</t>
-  </si>
-  <si>
-    <t>elc_won_010</t>
-  </si>
-  <si>
-    <t>rez_won_011</t>
-  </si>
-  <si>
-    <t>elc_won_011</t>
-  </si>
-  <si>
-    <t>rez_won_012</t>
-  </si>
-  <si>
-    <t>elc_won_012</t>
-  </si>
-  <si>
-    <t>rez_won_013</t>
-  </si>
-  <si>
-    <t>elc_won_013</t>
-  </si>
-  <si>
-    <t>rez_won_014</t>
-  </si>
-  <si>
-    <t>elc_won_014</t>
-  </si>
-  <si>
-    <t>rez_won_015</t>
-  </si>
-  <si>
-    <t>elc_won_015</t>
-  </si>
-  <si>
-    <t>rez_won_016</t>
-  </si>
-  <si>
-    <t>elc_won_016</t>
-  </si>
-  <si>
-    <t>rez_won_017</t>
-  </si>
-  <si>
-    <t>elc_won_017</t>
-  </si>
-  <si>
-    <t>rez_won_018</t>
-  </si>
-  <si>
-    <t>elc_won_018</t>
-  </si>
-  <si>
-    <t>rez_won_019</t>
-  </si>
-  <si>
-    <t>elc_won_019</t>
-  </si>
-  <si>
-    <t>rez_won_020</t>
-  </si>
-  <si>
-    <t>elc_won_020</t>
-  </si>
-  <si>
-    <t>rez_wof_001</t>
-  </si>
-  <si>
-    <t>elc_wof_001</t>
-  </si>
-  <si>
-    <t>rez_wof_002</t>
-  </si>
-  <si>
-    <t>elc_wof_002</t>
-  </si>
-  <si>
-    <t>rez_wof_003</t>
-  </si>
-  <si>
-    <t>elc_wof_003</t>
-  </si>
-  <si>
-    <t>rez_wof_004</t>
-  </si>
-  <si>
-    <t>elc_wof_004</t>
-  </si>
-  <si>
-    <t>rez_wof_005</t>
-  </si>
-  <si>
-    <t>elc_wof_005</t>
-  </si>
-  <si>
-    <t>rez_wof_006</t>
-  </si>
-  <si>
-    <t>elc_wof_006</t>
-  </si>
-  <si>
-    <t>rez_wof_007</t>
-  </si>
-  <si>
-    <t>elc_wof_007</t>
-  </si>
-  <si>
-    <t>rez_wof_008</t>
-  </si>
-  <si>
-    <t>elc_wof_008</t>
-  </si>
-  <si>
-    <t>rez_wof_009</t>
-  </si>
-  <si>
-    <t>elc_wof_009</t>
-  </si>
-  <si>
-    <t>rez_wof_010</t>
-  </si>
-  <si>
-    <t>elc_wof_010</t>
+    <t>p_PL10-400_POL</t>
+  </si>
+  <si>
+    <t>e_PL10-400_POL*</t>
+  </si>
+  <si>
+    <t>p_PL11-220_POL</t>
+  </si>
+  <si>
+    <t>e_PL11-220_POL*</t>
+  </si>
+  <si>
+    <t>p_PL11-400_POL</t>
+  </si>
+  <si>
+    <t>e_PL11-400_POL*</t>
+  </si>
+  <si>
+    <t>p_PL13-220_POL</t>
+  </si>
+  <si>
+    <t>e_PL13-220_POL*</t>
+  </si>
+  <si>
+    <t>p_PL13-400_POL</t>
+  </si>
+  <si>
+    <t>e_PL13-400_POL*</t>
+  </si>
+  <si>
+    <t>p_PL14-220_POL</t>
+  </si>
+  <si>
+    <t>e_PL14-220_POL*</t>
+  </si>
+  <si>
+    <t>p_PL14-400_POL</t>
+  </si>
+  <si>
+    <t>e_PL14-400_POL*</t>
+  </si>
+  <si>
+    <t>p_PL15-400_POL</t>
+  </si>
+  <si>
+    <t>e_PL15-400_POL*</t>
+  </si>
+  <si>
+    <t>p_PL16-400_POL</t>
+  </si>
+  <si>
+    <t>e_PL16-400_POL*</t>
+  </si>
+  <si>
+    <t>p_PL17-400_POL</t>
+  </si>
+  <si>
+    <t>e_PL17-400_POL*</t>
+  </si>
+  <si>
+    <t>p_PL18-400_POL</t>
+  </si>
+  <si>
+    <t>e_PL18-400_POL*</t>
+  </si>
+  <si>
+    <t>p_PL19-220_POL</t>
+  </si>
+  <si>
+    <t>e_PL19-220_POL*</t>
+  </si>
+  <si>
+    <t>p_PL2-220_POL</t>
+  </si>
+  <si>
+    <t>e_PL2-220_POL*</t>
+  </si>
+  <si>
+    <t>p_PL20-220_POL</t>
+  </si>
+  <si>
+    <t>e_PL20-220_POL*</t>
+  </si>
+  <si>
+    <t>p_PL21-220_POL</t>
+  </si>
+  <si>
+    <t>e_PL21-220_POL*</t>
+  </si>
+  <si>
+    <t>p_PL22-220_POL</t>
+  </si>
+  <si>
+    <t>e_PL22-220_POL*</t>
+  </si>
+  <si>
+    <t>p_PL23-400_POL</t>
+  </si>
+  <si>
+    <t>e_PL23-400_POL*</t>
+  </si>
+  <si>
+    <t>p_PL24-220_POL</t>
+  </si>
+  <si>
+    <t>e_PL24-220_POL*</t>
+  </si>
+  <si>
+    <t>p_PL25-220_POL</t>
+  </si>
+  <si>
+    <t>e_PL25-220_POL*</t>
+  </si>
+  <si>
+    <t>p_PL25-400_POL</t>
+  </si>
+  <si>
+    <t>e_PL25-400_POL*</t>
+  </si>
+  <si>
+    <t>p_PL26-400_POL</t>
+  </si>
+  <si>
+    <t>e_PL26-400_POL*</t>
+  </si>
+  <si>
+    <t>p_PL27-400_POL</t>
+  </si>
+  <si>
+    <t>e_PL27-400_POL*</t>
+  </si>
+  <si>
+    <t>p_PL28-400_POL</t>
+  </si>
+  <si>
+    <t>e_PL28-400_POL*</t>
+  </si>
+  <si>
+    <t>p_PL29-400_POL</t>
+  </si>
+  <si>
+    <t>e_PL29-400_POL*</t>
+  </si>
+  <si>
+    <t>p_PL3-220_POL</t>
+  </si>
+  <si>
+    <t>e_PL3-220_POL*</t>
+  </si>
+  <si>
+    <t>p_PL30-220_POL</t>
+  </si>
+  <si>
+    <t>e_PL30-220_POL*</t>
+  </si>
+  <si>
+    <t>p_PL31-400_POL</t>
+  </si>
+  <si>
+    <t>e_PL31-400_POL*</t>
+  </si>
+  <si>
+    <t>p_PL32-220_POL</t>
+  </si>
+  <si>
+    <t>e_PL32-220_POL*</t>
+  </si>
+  <si>
+    <t>p_PL33-220_POL</t>
+  </si>
+  <si>
+    <t>e_PL33-220_POL*</t>
+  </si>
+  <si>
+    <t>p_PL34-400_POL</t>
+  </si>
+  <si>
+    <t>e_PL34-400_POL*</t>
+  </si>
+  <si>
+    <t>p_PL35-220_POL</t>
+  </si>
+  <si>
+    <t>e_PL35-220_POL*</t>
+  </si>
+  <si>
+    <t>p_PL36-400_POL</t>
+  </si>
+  <si>
+    <t>e_PL36-400_POL*</t>
+  </si>
+  <si>
+    <t>p_PL37-220_POL</t>
+  </si>
+  <si>
+    <t>e_PL37-220_POL*</t>
+  </si>
+  <si>
+    <t>p_PL38-400_POL</t>
+  </si>
+  <si>
+    <t>e_PL38-400_POL*</t>
+  </si>
+  <si>
+    <t>p_PL39-220_POL</t>
+  </si>
+  <si>
+    <t>e_PL39-220_POL*</t>
+  </si>
+  <si>
+    <t>p_PL4-220_POL</t>
+  </si>
+  <si>
+    <t>e_PL4-220_POL*</t>
+  </si>
+  <si>
+    <t>p_PL40-220_POL</t>
+  </si>
+  <si>
+    <t>e_PL40-220_POL*</t>
+  </si>
+  <si>
+    <t>p_PL40-400_POL</t>
+  </si>
+  <si>
+    <t>e_PL40-400_POL*</t>
+  </si>
+  <si>
+    <t>p_PL41-400_POL</t>
+  </si>
+  <si>
+    <t>e_PL41-400_POL*</t>
+  </si>
+  <si>
+    <t>p_PL42-220_POL</t>
+  </si>
+  <si>
+    <t>e_PL42-220_POL*</t>
+  </si>
+  <si>
+    <t>p_PL43-220_POL</t>
+  </si>
+  <si>
+    <t>e_PL43-220_POL*</t>
+  </si>
+  <si>
+    <t>p_PL44-220_POL</t>
+  </si>
+  <si>
+    <t>e_PL44-220_POL*</t>
+  </si>
+  <si>
+    <t>p_PL45-220_POL</t>
+  </si>
+  <si>
+    <t>e_PL45-220_POL*</t>
+  </si>
+  <si>
+    <t>p_PL46-220_POL</t>
+  </si>
+  <si>
+    <t>e_PL46-220_POL*</t>
+  </si>
+  <si>
+    <t>p_PL47-220_POL</t>
+  </si>
+  <si>
+    <t>e_PL47-220_POL*</t>
+  </si>
+  <si>
+    <t>p_PL48-220_POL</t>
+  </si>
+  <si>
+    <t>e_PL48-220_POL*</t>
+  </si>
+  <si>
+    <t>p_PL49-220_POL</t>
+  </si>
+  <si>
+    <t>e_PL49-220_POL*</t>
+  </si>
+  <si>
+    <t>p_PL5-220_POL</t>
+  </si>
+  <si>
+    <t>e_PL5-220_POL*</t>
+  </si>
+  <si>
+    <t>p_PL50-220_POL</t>
+  </si>
+  <si>
+    <t>e_PL50-220_POL*</t>
+  </si>
+  <si>
+    <t>p_PL51-400_POL</t>
+  </si>
+  <si>
+    <t>e_PL51-400_POL*</t>
+  </si>
+  <si>
+    <t>p_PL52-400_POL</t>
+  </si>
+  <si>
+    <t>e_PL52-400_POL*</t>
+  </si>
+  <si>
+    <t>p_PL53-220_POL</t>
+  </si>
+  <si>
+    <t>e_PL53-220_POL*</t>
+  </si>
+  <si>
+    <t>p_PL54-220_POL</t>
+  </si>
+  <si>
+    <t>e_PL54-220_POL*</t>
+  </si>
+  <si>
+    <t>p_PL54-400_POL</t>
+  </si>
+  <si>
+    <t>e_PL54-400_POL*</t>
+  </si>
+  <si>
+    <t>p_PL55-220_POL</t>
+  </si>
+  <si>
+    <t>e_PL55-220_POL*</t>
+  </si>
+  <si>
+    <t>p_PL56-220_POL</t>
+  </si>
+  <si>
+    <t>e_PL56-220_POL*</t>
+  </si>
+  <si>
+    <t>p_PL57-220_POL</t>
+  </si>
+  <si>
+    <t>e_PL57-220_POL*</t>
+  </si>
+  <si>
+    <t>p_PL58-220_POL</t>
+  </si>
+  <si>
+    <t>e_PL58-220_POL*</t>
+  </si>
+  <si>
+    <t>p_PL59-220_POL</t>
+  </si>
+  <si>
+    <t>e_PL59-220_POL*</t>
+  </si>
+  <si>
+    <t>p_PL59-400_POL</t>
+  </si>
+  <si>
+    <t>e_PL59-400_POL*</t>
+  </si>
+  <si>
+    <t>p_PL6-220_POL</t>
+  </si>
+  <si>
+    <t>e_PL6-220_POL*</t>
+  </si>
+  <si>
+    <t>p_PL60-220_POL</t>
+  </si>
+  <si>
+    <t>e_PL60-220_POL*</t>
+  </si>
+  <si>
+    <t>p_PL61-220_POL</t>
+  </si>
+  <si>
+    <t>e_PL61-220_POL*</t>
+  </si>
+  <si>
+    <t>p_PL62-400_POL</t>
+  </si>
+  <si>
+    <t>e_PL62-400_POL*</t>
+  </si>
+  <si>
+    <t>p_PL7-400_POL</t>
+  </si>
+  <si>
+    <t>e_PL7-400_POL*</t>
+  </si>
+  <si>
+    <t>p_PL8-220_POL</t>
+  </si>
+  <si>
+    <t>e_PL8-220_POL*</t>
+  </si>
+  <si>
+    <t>p_r18085709-400_POL</t>
+  </si>
+  <si>
+    <t>e_r18085709-400_POL*</t>
+  </si>
+  <si>
+    <t>p_r9399771-220_POL</t>
+  </si>
+  <si>
+    <t>e_r9399771-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w101914781-220_POL</t>
+  </si>
+  <si>
+    <t>e_w101914781-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w101914781-400_POL</t>
+  </si>
+  <si>
+    <t>e_w101914781-400_POL*</t>
+  </si>
+  <si>
+    <t>p_w101915790-220_POL</t>
+  </si>
+  <si>
+    <t>e_w101915790-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w101982559-220_POL</t>
+  </si>
+  <si>
+    <t>e_w101982559-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w102165724-220_POL</t>
+  </si>
+  <si>
+    <t>e_w102165724-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w1022342082-220_POL</t>
+  </si>
+  <si>
+    <t>e_w1022342082-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w1022342082-400_POL</t>
+  </si>
+  <si>
+    <t>e_w1022342082-400_POL*</t>
+  </si>
+  <si>
+    <t>p_w111615226-220_POL</t>
+  </si>
+  <si>
+    <t>e_w111615226-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w111615226-380_POL</t>
+  </si>
+  <si>
+    <t>e_w111615226-380_POL*</t>
+  </si>
+  <si>
+    <t>p_w111615226-400_POL</t>
+  </si>
+  <si>
+    <t>e_w111615226-400_POL*</t>
+  </si>
+  <si>
+    <t>p_w112614319-400_POL</t>
+  </si>
+  <si>
+    <t>e_w112614319-400_POL*</t>
+  </si>
+  <si>
+    <t>p_w115801644-220_POL</t>
+  </si>
+  <si>
+    <t>e_w115801644-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w121656686-220_POL</t>
+  </si>
+  <si>
+    <t>e_w121656686-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w121656686-400_POL</t>
+  </si>
+  <si>
+    <t>e_w121656686-400_POL*</t>
+  </si>
+  <si>
+    <t>p_w130644710-220_POL</t>
+  </si>
+  <si>
+    <t>e_w130644710-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w130644710-400_POL</t>
+  </si>
+  <si>
+    <t>e_w130644710-400_POL*</t>
+  </si>
+  <si>
+    <t>p_w131120723-220_POL</t>
+  </si>
+  <si>
+    <t>e_w131120723-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w133537926-220_POL</t>
+  </si>
+  <si>
+    <t>e_w133537926-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w133537926-400_POL</t>
+  </si>
+  <si>
+    <t>e_w133537926-400_POL*</t>
+  </si>
+  <si>
+    <t>p_w135598292-220_POL</t>
+  </si>
+  <si>
+    <t>e_w135598292-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w139452056-220_POL</t>
+  </si>
+  <si>
+    <t>e_w139452056-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w139452056-400_POL</t>
+  </si>
+  <si>
+    <t>e_w139452056-400_POL*</t>
+  </si>
+  <si>
+    <t>p_w143484238-220_POL</t>
+  </si>
+  <si>
+    <t>e_w143484238-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w144646702-400_POL</t>
+  </si>
+  <si>
+    <t>e_w144646702-400_POL*</t>
+  </si>
+  <si>
+    <t>p_w145037309-220_POL</t>
+  </si>
+  <si>
+    <t>e_w145037309-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w148060965-400_POL</t>
+  </si>
+  <si>
+    <t>e_w148060965-400_POL*</t>
+  </si>
+  <si>
+    <t>p_w148197330-220_POL</t>
+  </si>
+  <si>
+    <t>e_w148197330-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w153838553-220_POL</t>
+  </si>
+  <si>
+    <t>e_w153838553-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w154510504-400_POL</t>
+  </si>
+  <si>
+    <t>e_w154510504-400_POL*</t>
+  </si>
+  <si>
+    <t>p_w154894455-400_POL</t>
+  </si>
+  <si>
+    <t>e_w154894455-400_POL*</t>
+  </si>
+  <si>
+    <t>p_w155971668-220_POL</t>
+  </si>
+  <si>
+    <t>e_w155971668-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w158232924-220_POL</t>
+  </si>
+  <si>
+    <t>e_w158232924-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w165763717-220_POL</t>
+  </si>
+  <si>
+    <t>e_w165763717-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w166710856-400_POL</t>
+  </si>
+  <si>
+    <t>e_w166710856-400_POL*</t>
+  </si>
+  <si>
+    <t>p_w166838338-400_POL</t>
+  </si>
+  <si>
+    <t>e_w166838338-400_POL*</t>
+  </si>
+  <si>
+    <t>p_w170249563-220_POL</t>
+  </si>
+  <si>
+    <t>e_w170249563-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w170259740-220_POL</t>
+  </si>
+  <si>
+    <t>e_w170259740-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w170316833-220_POL</t>
+  </si>
+  <si>
+    <t>e_w170316833-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w170368942-220_POL</t>
+  </si>
+  <si>
+    <t>e_w170368942-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w171383831-220_POL</t>
+  </si>
+  <si>
+    <t>e_w171383831-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w171917072-400_POL</t>
+  </si>
+  <si>
+    <t>e_w171917072-400_POL*</t>
+  </si>
+  <si>
+    <t>p_w171992870-220_POL</t>
+  </si>
+  <si>
+    <t>e_w171992870-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w173582810-220_POL</t>
+  </si>
+  <si>
+    <t>e_w173582810-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w173582810-400_POL</t>
+  </si>
+  <si>
+    <t>e_w173582810-400_POL*</t>
+  </si>
+  <si>
+    <t>p_w173613665-220_POL</t>
+  </si>
+  <si>
+    <t>e_w173613665-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w175406958-220_POL</t>
+  </si>
+  <si>
+    <t>e_w175406958-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w175406958-400_POL</t>
+  </si>
+  <si>
+    <t>e_w175406958-400_POL*</t>
+  </si>
+  <si>
+    <t>p_w177749653-220_POL</t>
+  </si>
+  <si>
+    <t>e_w177749653-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w178756295-220_POL</t>
+  </si>
+  <si>
+    <t>e_w178756295-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w178838661-220_POL</t>
+  </si>
+  <si>
+    <t>e_w178838661-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w178838661-400_POL</t>
+  </si>
+  <si>
+    <t>e_w178838661-400_POL*</t>
+  </si>
+  <si>
+    <t>p_w179279860-220_POL</t>
+  </si>
+  <si>
+    <t>e_w179279860-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w180535363-220_POL</t>
+  </si>
+  <si>
+    <t>e_w180535363-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w180542657-220_POL</t>
+  </si>
+  <si>
+    <t>e_w180542657-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w180542657-400_POL</t>
+  </si>
+  <si>
+    <t>e_w180542657-400_POL*</t>
+  </si>
+  <si>
+    <t>p_w183259405-220_POL</t>
+  </si>
+  <si>
+    <t>e_w183259405-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w183945016-220_POL</t>
+  </si>
+  <si>
+    <t>e_w183945016-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w184899160-220_POL</t>
+  </si>
+  <si>
+    <t>e_w184899160-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w185454704-220_POL</t>
+  </si>
+  <si>
+    <t>e_w185454704-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w185459155-220_POL</t>
+  </si>
+  <si>
+    <t>e_w185459155-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w189501431-220_POL</t>
+  </si>
+  <si>
+    <t>e_w189501431-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w189501431-400_POL</t>
+  </si>
+  <si>
+    <t>e_w189501431-400_POL*</t>
+  </si>
+  <si>
+    <t>p_w189851841-220_POL</t>
+  </si>
+  <si>
+    <t>e_w189851841-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w191035265-220_POL</t>
+  </si>
+  <si>
+    <t>e_w191035265-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w191038569-220_POL</t>
+  </si>
+  <si>
+    <t>e_w191038569-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w191352746-220_POL</t>
+  </si>
+  <si>
+    <t>e_w191352746-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w194903381-220_POL</t>
+  </si>
+  <si>
+    <t>e_w194903381-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w194903381-400_POL</t>
+  </si>
+  <si>
+    <t>e_w194903381-400_POL*</t>
+  </si>
+  <si>
+    <t>p_w198635989-220_POL</t>
+  </si>
+  <si>
+    <t>e_w198635989-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w199098050-220_POL</t>
+  </si>
+  <si>
+    <t>e_w199098050-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w199098050-400_POL</t>
+  </si>
+  <si>
+    <t>e_w199098050-400_POL*</t>
+  </si>
+  <si>
+    <t>p_w199098053-220_POL</t>
+  </si>
+  <si>
+    <t>e_w199098053-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w199098053-400_POL</t>
+  </si>
+  <si>
+    <t>e_w199098053-400_POL*</t>
+  </si>
+  <si>
+    <t>p_w199098055-220_POL</t>
+  </si>
+  <si>
+    <t>e_w199098055-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w215282393-400_POL</t>
+  </si>
+  <si>
+    <t>e_w215282393-400_POL*</t>
+  </si>
+  <si>
+    <t>p_w216060722-220_POL</t>
+  </si>
+  <si>
+    <t>e_w216060722-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w216975352-220_POL</t>
+  </si>
+  <si>
+    <t>e_w216975352-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w217899005-220_POL</t>
+  </si>
+  <si>
+    <t>e_w217899005-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w224727316-220_POL</t>
+  </si>
+  <si>
+    <t>e_w224727316-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w228154083-220_POL</t>
+  </si>
+  <si>
+    <t>e_w228154083-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w238640596-220_POL</t>
+  </si>
+  <si>
+    <t>e_w238640596-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w238640596-400_POL</t>
+  </si>
+  <si>
+    <t>e_w238640596-400_POL*</t>
+  </si>
+  <si>
+    <t>p_w241842600-220_POL</t>
+  </si>
+  <si>
+    <t>e_w241842600-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w241842600-400_POL</t>
+  </si>
+  <si>
+    <t>e_w241842600-400_POL*</t>
+  </si>
+  <si>
+    <t>p_w245964556-220_POL</t>
+  </si>
+  <si>
+    <t>e_w245964556-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w251239544-220_POL</t>
+  </si>
+  <si>
+    <t>e_w251239544-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w251239544-400_POL</t>
+  </si>
+  <si>
+    <t>e_w251239544-400_POL*</t>
+  </si>
+  <si>
+    <t>p_w254235846-220_POL</t>
+  </si>
+  <si>
+    <t>e_w254235846-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w254235846-400_POL</t>
+  </si>
+  <si>
+    <t>e_w254235846-400_POL*</t>
+  </si>
+  <si>
+    <t>p_w254938713-220_POL</t>
+  </si>
+  <si>
+    <t>e_w254938713-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w254938713-400_POL</t>
+  </si>
+  <si>
+    <t>e_w254938713-400_POL*</t>
+  </si>
+  <si>
+    <t>p_w255232597-220_POL</t>
+  </si>
+  <si>
+    <t>e_w255232597-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w255277953-400_POL</t>
+  </si>
+  <si>
+    <t>e_w255277953-400_POL*</t>
+  </si>
+  <si>
+    <t>p_w255284259-220_POL</t>
+  </si>
+  <si>
+    <t>e_w255284259-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w255284259-400_POL</t>
+  </si>
+  <si>
+    <t>e_w255284259-400_POL*</t>
+  </si>
+  <si>
+    <t>p_w255293400-220_POL</t>
+  </si>
+  <si>
+    <t>e_w255293400-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w255293400-400_POL</t>
+  </si>
+  <si>
+    <t>e_w255293400-400_POL*</t>
+  </si>
+  <si>
+    <t>p_w255293403-400_POL</t>
+  </si>
+  <si>
+    <t>e_w255293403-400_POL*</t>
+  </si>
+  <si>
+    <t>p_w255314292_POL</t>
+  </si>
+  <si>
+    <t>e_w255314292_POL*</t>
+  </si>
+  <si>
+    <t>p_w255972326-400_POL</t>
+  </si>
+  <si>
+    <t>e_w255972326-400_POL*</t>
+  </si>
+  <si>
+    <t>p_w255972397-400_POL</t>
+  </si>
+  <si>
+    <t>e_w255972397-400_POL*</t>
+  </si>
+  <si>
+    <t>p_w255973806-220_POL</t>
+  </si>
+  <si>
+    <t>e_w255973806-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w255973806-400_POL</t>
+  </si>
+  <si>
+    <t>e_w255973806-400_POL*</t>
+  </si>
+  <si>
+    <t>p_w25898810-220_POL</t>
+  </si>
+  <si>
+    <t>e_w25898810-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w276291999-220_POL</t>
+  </si>
+  <si>
+    <t>e_w276291999-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w276291999-400_POL</t>
+  </si>
+  <si>
+    <t>e_w276291999-400_POL*</t>
+  </si>
+  <si>
+    <t>p_w29098336-220_POL</t>
+  </si>
+  <si>
+    <t>e_w29098336-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w29115701-220_POL</t>
+  </si>
+  <si>
+    <t>e_w29115701-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w291375946-220_POL</t>
+  </si>
+  <si>
+    <t>e_w291375946-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w29139402-220_POL</t>
+  </si>
+  <si>
+    <t>e_w29139402-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w293484891-220_POL</t>
+  </si>
+  <si>
+    <t>e_w293484891-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w293484891-400_POL</t>
+  </si>
+  <si>
+    <t>e_w293484891-400_POL*</t>
+  </si>
+  <si>
+    <t>p_w293484894-220_POL</t>
+  </si>
+  <si>
+    <t>e_w293484894-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w293489607-400_POL</t>
+  </si>
+  <si>
+    <t>e_w293489607-400_POL*</t>
+  </si>
+  <si>
+    <t>p_w293489663-400_POL</t>
+  </si>
+  <si>
+    <t>e_w293489663-400_POL*</t>
+  </si>
+  <si>
+    <t>p_w303870256-400_POL</t>
+  </si>
+  <si>
+    <t>e_w303870256-400_POL*</t>
+  </si>
+  <si>
+    <t>p_w32036484-220_POL</t>
+  </si>
+  <si>
+    <t>e_w32036484-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w32036484-400_POL</t>
+  </si>
+  <si>
+    <t>e_w32036484-400_POL*</t>
+  </si>
+  <si>
+    <t>p_w32943179-220_POL</t>
+  </si>
+  <si>
+    <t>e_w32943179-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w32943179-400_POL</t>
+  </si>
+  <si>
+    <t>e_w32943179-400_POL*</t>
+  </si>
+  <si>
+    <t>p_w336990960-220_POL</t>
+  </si>
+  <si>
+    <t>e_w336990960-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w35366436-220_POL</t>
+  </si>
+  <si>
+    <t>e_w35366436-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w385098015-400_POL</t>
+  </si>
+  <si>
+    <t>e_w385098015-400_POL*</t>
+  </si>
+  <si>
+    <t>p_w385118244-400_POL</t>
+  </si>
+  <si>
+    <t>e_w385118244-400_POL*</t>
+  </si>
+  <si>
+    <t>p_w385539724-220_POL</t>
+  </si>
+  <si>
+    <t>e_w385539724-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w39428977-220_POL</t>
+  </si>
+  <si>
+    <t>e_w39428977-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w39428977-400_POL</t>
+  </si>
+  <si>
+    <t>e_w39428977-400_POL*</t>
+  </si>
+  <si>
+    <t>p_w40062974-220_POL</t>
+  </si>
+  <si>
+    <t>e_w40062974-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w40946784-400_POL</t>
+  </si>
+  <si>
+    <t>e_w40946784-400_POL*</t>
+  </si>
+  <si>
+    <t>p_w40946790-220_POL</t>
+  </si>
+  <si>
+    <t>e_w40946790-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w44389929-220_POL</t>
+  </si>
+  <si>
+    <t>e_w44389929-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w46092396-220_POL</t>
+  </si>
+  <si>
+    <t>e_w46092396-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w46092396-400_POL</t>
+  </si>
+  <si>
+    <t>e_w46092396-400_POL*</t>
+  </si>
+  <si>
+    <t>p_w46235456-220_POL</t>
+  </si>
+  <si>
+    <t>e_w46235456-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w46235456-400_POL</t>
+  </si>
+  <si>
+    <t>e_w46235456-400_POL*</t>
+  </si>
+  <si>
+    <t>p_w534238983-220_POL</t>
+  </si>
+  <si>
+    <t>e_w534238983-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w534238983-400_POL</t>
+  </si>
+  <si>
+    <t>e_w534238983-400_POL*</t>
+  </si>
+  <si>
+    <t>p_w658600169-400_POL</t>
+  </si>
+  <si>
+    <t>e_w658600169-400_POL*</t>
+  </si>
+  <si>
+    <t>p_w66051759-220_POL</t>
+  </si>
+  <si>
+    <t>e_w66051759-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w66161634-220_POL</t>
+  </si>
+  <si>
+    <t>e_w66161634-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w66161634-400_POL</t>
+  </si>
+  <si>
+    <t>e_w66161634-400_POL*</t>
+  </si>
+  <si>
+    <t>p_w668348943-220_POL</t>
+  </si>
+  <si>
+    <t>e_w668348943-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w681264796-220_POL</t>
+  </si>
+  <si>
+    <t>e_w681264796-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w681264796-400_POL</t>
+  </si>
+  <si>
+    <t>e_w681264796-400_POL*</t>
+  </si>
+  <si>
+    <t>p_w726776987-220_POL</t>
+  </si>
+  <si>
+    <t>e_w726776987-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w72879943-220_POL</t>
+  </si>
+  <si>
+    <t>e_w72879943-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w79033485-400_POL</t>
+  </si>
+  <si>
+    <t>e_w79033485-400_POL*</t>
+  </si>
+  <si>
+    <t>p_w86494356-400_POL</t>
+  </si>
+  <si>
+    <t>e_w86494356-400_POL*</t>
+  </si>
+  <si>
+    <t>p_w87667718-220_POL</t>
+  </si>
+  <si>
+    <t>e_w87667718-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w88544449-220_POL</t>
+  </si>
+  <si>
+    <t>e_w88544449-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w89434732-220_POL</t>
+  </si>
+  <si>
+    <t>e_w89434732-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w91384044-400_POL</t>
+  </si>
+  <si>
+    <t>e_w91384044-400_POL*</t>
+  </si>
+  <si>
+    <t>p_w98611253-220_POL</t>
+  </si>
+  <si>
+    <t>e_w98611253-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w98634956-220_POL</t>
+  </si>
+  <si>
+    <t>e_w98634956-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w99593626-220_POL</t>
+  </si>
+  <si>
+    <t>e_w99593626-220_POL*</t>
+  </si>
+  <si>
+    <t>p_w99593626-400_POL</t>
+  </si>
+  <si>
+    <t>e_w99593626-400_POL*</t>
+  </si>
+  <si>
+    <t>rez_spv_POL_001</t>
+  </si>
+  <si>
+    <t>elc_spv_POL_001</t>
+  </si>
+  <si>
+    <t>rez_spv_POL_002</t>
+  </si>
+  <si>
+    <t>elc_spv_POL_002</t>
+  </si>
+  <si>
+    <t>rez_spv_POL_003</t>
+  </si>
+  <si>
+    <t>elc_spv_POL_003</t>
+  </si>
+  <si>
+    <t>rez_spv_POL_004</t>
+  </si>
+  <si>
+    <t>elc_spv_POL_004</t>
+  </si>
+  <si>
+    <t>rez_spv_POL_005</t>
+  </si>
+  <si>
+    <t>elc_spv_POL_005</t>
+  </si>
+  <si>
+    <t>rez_spv_POL_006</t>
+  </si>
+  <si>
+    <t>elc_spv_POL_006</t>
+  </si>
+  <si>
+    <t>rez_spv_POL_007</t>
+  </si>
+  <si>
+    <t>elc_spv_POL_007</t>
+  </si>
+  <si>
+    <t>rez_spv_POL_008</t>
+  </si>
+  <si>
+    <t>elc_spv_POL_008</t>
+  </si>
+  <si>
+    <t>rez_spv_POL_009</t>
+  </si>
+  <si>
+    <t>elc_spv_POL_009</t>
+  </si>
+  <si>
+    <t>rez_spv_POL_010</t>
+  </si>
+  <si>
+    <t>elc_spv_POL_010</t>
+  </si>
+  <si>
+    <t>rez_spv_POL_011</t>
+  </si>
+  <si>
+    <t>elc_spv_POL_011</t>
+  </si>
+  <si>
+    <t>rez_spv_POL_012</t>
+  </si>
+  <si>
+    <t>elc_spv_POL_012</t>
+  </si>
+  <si>
+    <t>rez_spv_POL_013</t>
+  </si>
+  <si>
+    <t>elc_spv_POL_013</t>
+  </si>
+  <si>
+    <t>rez_spv_POL_014</t>
+  </si>
+  <si>
+    <t>elc_spv_POL_014</t>
+  </si>
+  <si>
+    <t>rez_spv_POL_015</t>
+  </si>
+  <si>
+    <t>elc_spv_POL_015</t>
+  </si>
+  <si>
+    <t>rez_spv_POL_016</t>
+  </si>
+  <si>
+    <t>elc_spv_POL_016</t>
+  </si>
+  <si>
+    <t>rez_spv_POL_017</t>
+  </si>
+  <si>
+    <t>elc_spv_POL_017</t>
+  </si>
+  <si>
+    <t>rez_spv_POL_018</t>
+  </si>
+  <si>
+    <t>elc_spv_POL_018</t>
+  </si>
+  <si>
+    <t>rez_spv_POL_019</t>
+  </si>
+  <si>
+    <t>elc_spv_POL_019</t>
+  </si>
+  <si>
+    <t>rez_spv_POL_020</t>
+  </si>
+  <si>
+    <t>elc_spv_POL_020</t>
+  </si>
+  <si>
+    <t>rez_won_POL_001</t>
+  </si>
+  <si>
+    <t>elc_won_POL_001</t>
+  </si>
+  <si>
+    <t>rez_won_POL_002</t>
+  </si>
+  <si>
+    <t>elc_won_POL_002</t>
+  </si>
+  <si>
+    <t>rez_won_POL_003</t>
+  </si>
+  <si>
+    <t>elc_won_POL_003</t>
+  </si>
+  <si>
+    <t>rez_won_POL_004</t>
+  </si>
+  <si>
+    <t>elc_won_POL_004</t>
+  </si>
+  <si>
+    <t>rez_won_POL_005</t>
+  </si>
+  <si>
+    <t>elc_won_POL_005</t>
+  </si>
+  <si>
+    <t>rez_won_POL_006</t>
+  </si>
+  <si>
+    <t>elc_won_POL_006</t>
+  </si>
+  <si>
+    <t>rez_won_POL_007</t>
+  </si>
+  <si>
+    <t>elc_won_POL_007</t>
+  </si>
+  <si>
+    <t>rez_won_POL_008</t>
+  </si>
+  <si>
+    <t>elc_won_POL_008</t>
+  </si>
+  <si>
+    <t>rez_won_POL_009</t>
+  </si>
+  <si>
+    <t>elc_won_POL_009</t>
+  </si>
+  <si>
+    <t>rez_won_POL_010</t>
+  </si>
+  <si>
+    <t>elc_won_POL_010</t>
+  </si>
+  <si>
+    <t>rez_won_POL_011</t>
+  </si>
+  <si>
+    <t>elc_won_POL_011</t>
+  </si>
+  <si>
+    <t>rez_won_POL_012</t>
+  </si>
+  <si>
+    <t>elc_won_POL_012</t>
+  </si>
+  <si>
+    <t>rez_won_POL_013</t>
+  </si>
+  <si>
+    <t>elc_won_POL_013</t>
+  </si>
+  <si>
+    <t>rez_won_POL_014</t>
+  </si>
+  <si>
+    <t>elc_won_POL_014</t>
+  </si>
+  <si>
+    <t>rez_won_POL_015</t>
+  </si>
+  <si>
+    <t>elc_won_POL_015</t>
+  </si>
+  <si>
+    <t>rez_won_POL_016</t>
+  </si>
+  <si>
+    <t>elc_won_POL_016</t>
+  </si>
+  <si>
+    <t>rez_won_POL_017</t>
+  </si>
+  <si>
+    <t>elc_won_POL_017</t>
+  </si>
+  <si>
+    <t>rez_won_POL_018</t>
+  </si>
+  <si>
+    <t>elc_won_POL_018</t>
+  </si>
+  <si>
+    <t>rez_won_POL_019</t>
+  </si>
+  <si>
+    <t>elc_won_POL_019</t>
+  </si>
+  <si>
+    <t>rez_won_POL_020</t>
+  </si>
+  <si>
+    <t>elc_won_POL_020</t>
+  </si>
+  <si>
+    <t>rez_wof_POL_001</t>
+  </si>
+  <si>
+    <t>elc_wof_POL_001</t>
+  </si>
+  <si>
+    <t>rez_wof_POL_002</t>
+  </si>
+  <si>
+    <t>elc_wof_POL_002</t>
+  </si>
+  <si>
+    <t>rez_wof_POL_003</t>
+  </si>
+  <si>
+    <t>elc_wof_POL_003</t>
+  </si>
+  <si>
+    <t>rez_wof_POL_004</t>
+  </si>
+  <si>
+    <t>elc_wof_POL_004</t>
+  </si>
+  <si>
+    <t>rez_wof_POL_005</t>
+  </si>
+  <si>
+    <t>elc_wof_POL_005</t>
+  </si>
+  <si>
+    <t>rez_wof_POL_006</t>
+  </si>
+  <si>
+    <t>elc_wof_POL_006</t>
+  </si>
+  <si>
+    <t>rez_wof_POL_007</t>
+  </si>
+  <si>
+    <t>elc_wof_POL_007</t>
+  </si>
+  <si>
+    <t>rez_wof_POL_008</t>
+  </si>
+  <si>
+    <t>elc_wof_POL_008</t>
+  </si>
+  <si>
+    <t>rez_wof_POL_009</t>
+  </si>
+  <si>
+    <t>elc_wof_POL_009</t>
+  </si>
+  <si>
+    <t>rez_wof_POL_010</t>
+  </si>
+  <si>
+    <t>elc_wof_POL_010</t>
   </si>
 </sst>
 </file>
@@ -2585,8 +2837,8 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{09664D0A-6D44-49AF-97C0-9301A8143B6D}">
-  <dimension ref="B9:E243"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2ECA1A3A-3C8D-4F87-87CF-17F662BBDA27}">
+  <dimension ref="B9:E285"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
     <row r="9" spans="2:5" x14ac:dyDescent="0.45">
@@ -5867,6 +6119,594 @@
         <v>569</v>
       </c>
       <c r="E243" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="244" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B244" t="s">
+        <v>570</v>
+      </c>
+      <c r="C244" t="s">
+        <v>571</v>
+      </c>
+      <c r="D244" t="s">
+        <v>571</v>
+      </c>
+      <c r="E244" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="245" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B245" t="s">
+        <v>572</v>
+      </c>
+      <c r="C245" t="s">
+        <v>573</v>
+      </c>
+      <c r="D245" t="s">
+        <v>573</v>
+      </c>
+      <c r="E245" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="246" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B246" t="s">
+        <v>574</v>
+      </c>
+      <c r="C246" t="s">
+        <v>575</v>
+      </c>
+      <c r="D246" t="s">
+        <v>575</v>
+      </c>
+      <c r="E246" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="247" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B247" t="s">
+        <v>576</v>
+      </c>
+      <c r="C247" t="s">
+        <v>577</v>
+      </c>
+      <c r="D247" t="s">
+        <v>577</v>
+      </c>
+      <c r="E247" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="248" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B248" t="s">
+        <v>578</v>
+      </c>
+      <c r="C248" t="s">
+        <v>579</v>
+      </c>
+      <c r="D248" t="s">
+        <v>579</v>
+      </c>
+      <c r="E248" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="249" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B249" t="s">
+        <v>580</v>
+      </c>
+      <c r="C249" t="s">
+        <v>581</v>
+      </c>
+      <c r="D249" t="s">
+        <v>581</v>
+      </c>
+      <c r="E249" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="250" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B250" t="s">
+        <v>582</v>
+      </c>
+      <c r="C250" t="s">
+        <v>583</v>
+      </c>
+      <c r="D250" t="s">
+        <v>583</v>
+      </c>
+      <c r="E250" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="251" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B251" t="s">
+        <v>584</v>
+      </c>
+      <c r="C251" t="s">
+        <v>585</v>
+      </c>
+      <c r="D251" t="s">
+        <v>585</v>
+      </c>
+      <c r="E251" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="252" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B252" t="s">
+        <v>586</v>
+      </c>
+      <c r="C252" t="s">
+        <v>587</v>
+      </c>
+      <c r="D252" t="s">
+        <v>587</v>
+      </c>
+      <c r="E252" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="253" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B253" t="s">
+        <v>588</v>
+      </c>
+      <c r="C253" t="s">
+        <v>589</v>
+      </c>
+      <c r="D253" t="s">
+        <v>589</v>
+      </c>
+      <c r="E253" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="254" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B254" t="s">
+        <v>590</v>
+      </c>
+      <c r="C254" t="s">
+        <v>591</v>
+      </c>
+      <c r="D254" t="s">
+        <v>591</v>
+      </c>
+      <c r="E254" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="255" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B255" t="s">
+        <v>592</v>
+      </c>
+      <c r="C255" t="s">
+        <v>593</v>
+      </c>
+      <c r="D255" t="s">
+        <v>593</v>
+      </c>
+      <c r="E255" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="256" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B256" t="s">
+        <v>594</v>
+      </c>
+      <c r="C256" t="s">
+        <v>595</v>
+      </c>
+      <c r="D256" t="s">
+        <v>595</v>
+      </c>
+      <c r="E256" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="257" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B257" t="s">
+        <v>596</v>
+      </c>
+      <c r="C257" t="s">
+        <v>597</v>
+      </c>
+      <c r="D257" t="s">
+        <v>597</v>
+      </c>
+      <c r="E257" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="258" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B258" t="s">
+        <v>598</v>
+      </c>
+      <c r="C258" t="s">
+        <v>599</v>
+      </c>
+      <c r="D258" t="s">
+        <v>599</v>
+      </c>
+      <c r="E258" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="259" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B259" t="s">
+        <v>600</v>
+      </c>
+      <c r="C259" t="s">
+        <v>601</v>
+      </c>
+      <c r="D259" t="s">
+        <v>601</v>
+      </c>
+      <c r="E259" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="260" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B260" t="s">
+        <v>602</v>
+      </c>
+      <c r="C260" t="s">
+        <v>603</v>
+      </c>
+      <c r="D260" t="s">
+        <v>603</v>
+      </c>
+      <c r="E260" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="261" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B261" t="s">
+        <v>604</v>
+      </c>
+      <c r="C261" t="s">
+        <v>605</v>
+      </c>
+      <c r="D261" t="s">
+        <v>605</v>
+      </c>
+      <c r="E261" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="262" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B262" t="s">
+        <v>606</v>
+      </c>
+      <c r="C262" t="s">
+        <v>607</v>
+      </c>
+      <c r="D262" t="s">
+        <v>607</v>
+      </c>
+      <c r="E262" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="263" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B263" t="s">
+        <v>608</v>
+      </c>
+      <c r="C263" t="s">
+        <v>609</v>
+      </c>
+      <c r="D263" t="s">
+        <v>609</v>
+      </c>
+      <c r="E263" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="264" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B264" t="s">
+        <v>610</v>
+      </c>
+      <c r="C264" t="s">
+        <v>611</v>
+      </c>
+      <c r="D264" t="s">
+        <v>611</v>
+      </c>
+      <c r="E264" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="265" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B265" t="s">
+        <v>612</v>
+      </c>
+      <c r="C265" t="s">
+        <v>613</v>
+      </c>
+      <c r="D265" t="s">
+        <v>613</v>
+      </c>
+      <c r="E265" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="266" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B266" t="s">
+        <v>614</v>
+      </c>
+      <c r="C266" t="s">
+        <v>615</v>
+      </c>
+      <c r="D266" t="s">
+        <v>615</v>
+      </c>
+      <c r="E266" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="267" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B267" t="s">
+        <v>616</v>
+      </c>
+      <c r="C267" t="s">
+        <v>617</v>
+      </c>
+      <c r="D267" t="s">
+        <v>617</v>
+      </c>
+      <c r="E267" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="268" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B268" t="s">
+        <v>618</v>
+      </c>
+      <c r="C268" t="s">
+        <v>619</v>
+      </c>
+      <c r="D268" t="s">
+        <v>619</v>
+      </c>
+      <c r="E268" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="269" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B269" t="s">
+        <v>620</v>
+      </c>
+      <c r="C269" t="s">
+        <v>621</v>
+      </c>
+      <c r="D269" t="s">
+        <v>621</v>
+      </c>
+      <c r="E269" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="270" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B270" t="s">
+        <v>622</v>
+      </c>
+      <c r="C270" t="s">
+        <v>623</v>
+      </c>
+      <c r="D270" t="s">
+        <v>623</v>
+      </c>
+      <c r="E270" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="271" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B271" t="s">
+        <v>624</v>
+      </c>
+      <c r="C271" t="s">
+        <v>625</v>
+      </c>
+      <c r="D271" t="s">
+        <v>625</v>
+      </c>
+      <c r="E271" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="272" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B272" t="s">
+        <v>626</v>
+      </c>
+      <c r="C272" t="s">
+        <v>627</v>
+      </c>
+      <c r="D272" t="s">
+        <v>627</v>
+      </c>
+      <c r="E272" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="273" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B273" t="s">
+        <v>628</v>
+      </c>
+      <c r="C273" t="s">
+        <v>629</v>
+      </c>
+      <c r="D273" t="s">
+        <v>629</v>
+      </c>
+      <c r="E273" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="274" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B274" t="s">
+        <v>630</v>
+      </c>
+      <c r="C274" t="s">
+        <v>631</v>
+      </c>
+      <c r="D274" t="s">
+        <v>631</v>
+      </c>
+      <c r="E274" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="275" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B275" t="s">
+        <v>632</v>
+      </c>
+      <c r="C275" t="s">
+        <v>633</v>
+      </c>
+      <c r="D275" t="s">
+        <v>633</v>
+      </c>
+      <c r="E275" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="276" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B276" t="s">
+        <v>634</v>
+      </c>
+      <c r="C276" t="s">
+        <v>635</v>
+      </c>
+      <c r="D276" t="s">
+        <v>635</v>
+      </c>
+      <c r="E276" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="277" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B277" t="s">
+        <v>636</v>
+      </c>
+      <c r="C277" t="s">
+        <v>637</v>
+      </c>
+      <c r="D277" t="s">
+        <v>637</v>
+      </c>
+      <c r="E277" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="278" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B278" t="s">
+        <v>638</v>
+      </c>
+      <c r="C278" t="s">
+        <v>639</v>
+      </c>
+      <c r="D278" t="s">
+        <v>639</v>
+      </c>
+      <c r="E278" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="279" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B279" t="s">
+        <v>640</v>
+      </c>
+      <c r="C279" t="s">
+        <v>641</v>
+      </c>
+      <c r="D279" t="s">
+        <v>641</v>
+      </c>
+      <c r="E279" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="280" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B280" t="s">
+        <v>642</v>
+      </c>
+      <c r="C280" t="s">
+        <v>643</v>
+      </c>
+      <c r="D280" t="s">
+        <v>643</v>
+      </c>
+      <c r="E280" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="281" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B281" t="s">
+        <v>644</v>
+      </c>
+      <c r="C281" t="s">
+        <v>645</v>
+      </c>
+      <c r="D281" t="s">
+        <v>645</v>
+      </c>
+      <c r="E281" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="282" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B282" t="s">
+        <v>646</v>
+      </c>
+      <c r="C282" t="s">
+        <v>647</v>
+      </c>
+      <c r="D282" t="s">
+        <v>647</v>
+      </c>
+      <c r="E282" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="283" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B283" t="s">
+        <v>648</v>
+      </c>
+      <c r="C283" t="s">
+        <v>649</v>
+      </c>
+      <c r="D283" t="s">
+        <v>649</v>
+      </c>
+      <c r="E283" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="284" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B284" t="s">
+        <v>650</v>
+      </c>
+      <c r="C284" t="s">
+        <v>651</v>
+      </c>
+      <c r="D284" t="s">
+        <v>651</v>
+      </c>
+      <c r="E284" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="285" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B285" t="s">
+        <v>652</v>
+      </c>
+      <c r="C285" t="s">
+        <v>653</v>
+      </c>
+      <c r="D285" t="s">
+        <v>653</v>
+      </c>
+      <c r="E285" t="s">
         <v>105</v>
       </c>
     </row>

</xml_diff>